<commit_message>
added new data to Policia de Puerto Rico and modify observeEvent in server for minorities like Mujeres trans, Hombres trans, no binario and desconocido
</commit_message>
<xml_diff>
--- a/data/Negociado_de_Policia/nppr_maltrato.xlsx
+++ b/data/Negociado_de_Policia/nppr_maltrato.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orlando.hernandez\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Negociado_de_Policia\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41DA312F-5506-4125-8B36-F8CF4D3FD3BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435" activeTab="3"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2021" sheetId="1" r:id="rId1"/>
@@ -18,17 +19,28 @@
     <sheet name="2024" sheetId="4" r:id="rId4"/>
     <sheet name="2025" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="14">
   <si>
     <t>Tipo de Maltrato</t>
   </si>
@@ -64,12 +76,18 @@
   </si>
   <si>
     <t>Desconocido</t>
+  </si>
+  <si>
+    <t>Mujer Trans</t>
+  </si>
+  <si>
+    <t>No Binario</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -380,15 +398,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -399,7 +417,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -410,7 +428,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -421,7 +439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -432,7 +450,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -443,7 +461,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -454,7 +472,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -465,7 +483,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -482,15 +500,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -501,7 +519,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -512,7 +530,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -523,7 +541,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -534,7 +552,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -545,7 +563,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -556,7 +574,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -567,7 +585,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -584,15 +602,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -603,7 +621,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -614,7 +632,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -625,7 +643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -636,7 +654,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -647,7 +665,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -658,7 +676,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -669,7 +687,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -686,17 +704,18 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -713,7 +732,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -730,7 +749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -747,7 +766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -764,7 +783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -781,7 +800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -798,7 +817,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -815,7 +834,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -838,17 +857,19 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -859,21 +880,27 @@
         <v>9</v>
       </c>
       <c r="D1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" t="s">
         <v>10</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2">
-        <v>261</v>
+        <v>695</v>
       </c>
       <c r="C2">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -881,33 +908,45 @@
       <c r="E2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3">
-        <v>27</v>
+        <v>79</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
       <c r="B4">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -915,72 +954,102 @@
       <c r="E4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
       <c r="B5">
-        <v>297</v>
+        <v>724</v>
       </c>
       <c r="C5">
-        <v>47</v>
+        <v>125</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
       <c r="B6">
-        <v>1564</v>
+        <v>4128</v>
       </c>
       <c r="C6">
-        <v>249</v>
+        <v>767</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E6">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
       <c r="B7">
-        <v>867</v>
+        <v>2268</v>
       </c>
       <c r="C7">
-        <v>261</v>
+        <v>740</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
       <c r="B8">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
         <v>0</v>
       </c>
     </row>

</xml_diff>